<commit_message>
Align Product Card Variant mockup and RDS RQM with the current Quick setup.
Rename Settings.html, add GitHub Pages redirect, and document Enable custom, variant-as-product, and option sources so spec matches the Polariss mockup.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/RDS_Findter_Product_Card_Variant_RQM.xlsx
+++ b/docs/RDS_Findter_Product_Card_Variant_RQM.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="117">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -38,6 +38,22 @@
   </si>
   <si>
     <t xml:space="preserve">18/9/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cập nhật RQM theo mockup Settings.html mới.
+- Feature toggle đổi label thành Enable custom. Nested Options on card + Card behavior disable (không ẩn) khi OFF.
+- Thêm Show each variant as its own product: Collection/Search hiện 1 card / variant, ẩn option picker trên card.
+- Options on card thành bảng # / Option / Display / Show / Remove; Include all, Exclude all; kéo thả reorder; đổi option mapping trên row.
+- Merchant Add variant từ Shopify product option, Product metafield, hoặc Create custom option (display-only, không tạo SKU Shopify).
+- Preview bỏ Desktop/Mobile. Variant-as-product hiện 2 card split kèm variant title.
+- Save chuyển lên page header (nút Save). Display type trên Quick setup: Image swatch / Color swatch / Text button / Not shown.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mockup: findter-mockup/Settings.html
+Live: https://hainx-bss.github.io/Settings/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Done</t>
   </si>
   <si>
     <t xml:space="preserve">Rewrite RQM theo format RDS Findter (Changes Log / Admin Logic / Admin UI / StoreFront UI).
@@ -49,9 +65,6 @@
 Mockup: Settings.html / https://hainx-bss.github.io/Settings/</t>
   </si>
   <si>
-    <t xml:space="preserve">Done</t>
-  </si>
-  <si>
     <t xml:space="preserve">17/9/2026</t>
   </si>
   <si>
@@ -66,7 +79,7 @@
   <si>
     <t xml:space="preserve">Refine variant card settings and responsive preview.
 - Overflow +N đo theo width thật của card, không cắt giữa chip (fix XL / Wool).
-- Preview Desktop / Mobile.
+- Preview Desktop / Mobile (đã bỏ trên mockup 18/9/2026).
 - Ẩn UI legacy Variant Sets (max sets, hover source) khỏi mockup đang demo.</t>
   </si>
   <si>
@@ -79,115 +92,132 @@
     <t xml:space="preserve">Rename mockup page to Settings. Add Findter Filter &amp; Search mockup cho Product grid design.</t>
   </si>
   <si>
-    <t xml:space="preserve">Product Card Variant Options / Admin behavior</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Code UI/UX tham khảo: Settings.html
-Live mockup: https://hainx-bss.github.io/Settings/
-Format gốc: RDS_Findter_Merged_Filter_RQM.xlsx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI web tham khảo:
-https://hainx-bss.github.io/Settings/</t>
-  </si>
-  <si>
     <t xml:space="preserve">Logic requirement</t>
   </si>
   <si>
     <t xml:space="preserve">Mục tiêu
-- Merchant cấu hình variant options hiển thị trên product card (Collection / Search Result) mà không làm vỡ grid, đặc biệt trên mobile.
-- Admin Preview phải mô phỏng đúng presentation của storefront: display type, thứ tự option, overflow, swatch shape, click action.
-- Hệ thống hỗ trợ option name custom (Finish, Pack Size, Pattern…), không hard-code Color / Size / Material.
-- Availability và combination phải lấy từ variant data thật của Shopify, không từ scenario giả trong admin preview.
-- Save chỉ persist configuration của app. Không mutate product / variant data trên Shopify.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mockup: Settings.html
-Live: https://hainx-bss.github.io/Settings/</t>
+- Merchant cấu hình variant options trên product card (Collection / Search Result) mà không làm vỡ grid, đặc biệt trên mobile.
+- Có 2 presentation mode trên grid:
+  1) Product card + option picker (Enable custom ON, Show each variant as its own product OFF).
+  2) Mỗi variant là một product card riêng (Show each variant as its own product ON) — không hiện option picker trên card.
+- Admin Preview phải mô phỏng presentation storefront: display type, thứ tự option, overflow, swatch shape, click action, và split-card khi variant-as-product.
+- Option trên card lấy từ 3 source: Shopify product option, Product metafield, Custom option (app, display-only).
+- Không hard-code Color / Size / Material. Hỗ trợ option name bất kỳ (Finish, Pack Size, Pattern…).
+- Availability và combination purchasable lấy từ variant data thật của Shopify. Custom/metafield không tự tạo SKU mới.
+- Save chỉ persist configuration của app. Không mutate product / variant / option trên Shopify.</t>
   </si>
   <si>
     <t xml:space="preserve">Phạm vi áp dụng
 - Surface: product card trên Collection page và Search Result page.
-- Variant selection trên card phải tương thích với PDP Variant Picker và Quick Add.
-- Không áp dụng các setting này cho Variant Picker trên Product Detail Page.
-- Filter design (tab khác trên cùng màn Settings) nằm ngoài scope của RQM này.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Scope card only — không đổi PDP picker</t>
+- Variant selection trên card (mode option picker) phải tương thích với PDP Variant Picker và Quick Add.
+- Không áp dụng các setting option picker cho Variant Picker trên Product Detail Page.
+- Filter design (tab khác trên cùng màn Filter &amp; product grid design) nằm ngoài scope của RQM này.
+- Mode Show each variant as its own product chỉ đổi cách listing card trên Collection/Search, không đổi PDP.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scope card / collection grid — không đổi PDP picker</t>
   </si>
   <si>
     <t xml:space="preserve">Nguồn dữ liệu (source of truth)
-- Option list, option values, variant id, availability, media mapping đều import từ Shopify product/variant.
-- Màn hình này không cho merchant tạo option mới hoặc tạo value mới.
-- Mỗi Shopify source option là một Variant Set độc lập (ví dụ Color, Size, Material, Finish, Pack Size).
-- Unique key của value là option value id / variant id, không dùng display label.
-- Một source option chỉ được map vào đúng một Variant Set. Cấm map trùng.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Không hard-code Color/Size/Material</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cấu trúc dữ liệu tối thiểu của một Variant Set
-- sourceOptionId / sourceOptionName
-- enabled = true/false
-- presentationOrder (thứ tự trên card; chỉ ảnh hưởng presentation, không đổi Shopify option position)
-- displayType = Image swatch | Color swatch | Text button | Dropdown | Not shown
-- swatchShape = Circle | Square | Rounded (chỉ áp dụng Image/Color swatch)
-- imageSource = option value image | variant featured image | manual image (chỉ Image swatch)
-- clickBehavior = Update image and link | Open Quick Add | Open PDP
-- overflowMode = Show +N more (single line) | Horizontal scroll
-- unavailableStyle = Grey out | Hide | Cross out</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Click / overflow / unavailable đang là setting dùng chung cho mọi option trên card (theo mockup hiện tại).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Feature toggle: Enable variant options
-- Default an toàn: OFF. Khi OFF, product card không render bất kỳ option row nào.
-- Khi ON, chỉ render các option đang enabled, có source hợp lệ, và có visible value count &gt; 0.
-- Bật toggle trên product không có variant option: không render row rỗng.
-- Tắt/bật feature không được làm mất cấu hình đã lưu và không được đổi variant data Shopify.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADM-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Imported option list
-- Hiển thị đúng các option có thật trong variant data của catalog (ví dụ Color, Size, Material, Finish, Pack Size).
-- Hiện số values detected trên từng row.
-- Option bị xóa khỏi product sau sync: chuyển Needs attention hoặc ẩn, không giữ configuration rỗng trên storefront.
-- Data sync lỗi: giữ last known configuration; không render option không còn source.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADM-02 / LOG-01 / VAL-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Enable từng option + priority
-- Chỉ option đang bật mới vào candidate list để render trên card.
-- Option không có value hợp lệ: không render dù đang bật.
-- Drag &amp; drop đổi presentationOrder. Thứ tự này dùng cho card và cho việc ưu tiên khi không gian hẹp.
-- Drag không hợp lệ: giữ thứ tự cũ, không mất cấu hình.
-- Priority không đổi Shopify option position.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADM-03 / ADM-04</t>
+- Shopify product option: option list, values, variant id, availability, media mapping import từ Shopify. Values sync catalog và có thể resolve thành variant mua được.
+- Product metafield: dùng khi attribute không phải Shopify option. Phù hợp display / filter. Không tự tạo SKU mới.
+- Custom option: merchant tạo tên option display-only trên card. Không tạo Shopify option/value/variant. Khách không mua được combination không tồn tại.
+- Unique key của value là option value id / metafield value id / custom value id, không dùng display label.
+- Một Shopify option hoặc metafield chỉ được map vào đúng một row trên Options on card. Cấm map trùng.
+- Custom option key do app generate, không trùng catalog key.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Không hard-code Color/Size/Material
+Custom/metafield ≠ SKU mới</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cấu trúc dữ liệu tối thiểu
+Feature-level:
+- enableCustom = true/false (UI: Enable custom)
+- variantAsProduct = true/false (UI: Show each variant as its own product)
+- swatchShape = Circle | Square | Rounded (card-level, chỉ Image/Color swatch)
+- clickBehavior = Update image and link | Open quick add | Open product page (card-level)
+- overflowMode = Show +N more (single line) | Horizontal scroll (card-level)
+- unavailableStyle = Grey out | Hide | Cross out (card-level)
+Mỗi option row:
+- sourceType = product_option | metafield | custom
+- sourceKey / sourceName (và metafield namespace.key nếu có)
+- shown = true/false
+- presentationOrder (chỉ presentation, không đổi Shopify option position)
+- displayType = Image swatch | Color swatch | Text button | Not shown
+Dropdown display type không còn trên Quick setup mockup hiện tại. Image source (option value image / variant featured image / upload) chỉ còn trong legacy editor ẩn.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Click / overflow / unavailable / swatch shape là setting dùng chung cho mọi option trên card.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feature toggle: Enable custom
+- Label UI: Enable custom. Intro: Turn this on to show variant options on product cards, then choose which options appear.
+- Default an toàn production: OFF. Mockup demo đang ON.
+- Khi OFF: product card không render option row. Preview ẩn option. Nested panel Options on card + Card behavior disable (opacity + không tương tác), không ẩn hẳn để merchant vẫn thấy cấu trúc.
+- Khi ON và variantAsProduct OFF: render các option đang shown, display ≠ Not shown, source hợp lệ, visible value count &gt; 0.
+- Bật trên product không có variant option: không render row rỗng.
+- Tắt/bật không được làm mất cấu hình đã lưu và không được đổi variant data Shopify.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADM-01
+Mockup: #featureEnableToggle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mode: Show each variant as its own product
+- Toggle riêng, default OFF.
+- Helper: Collection and search show one card per variant instead of one card per product.
+- Khi ON: grid hiện 1 card / variant (ảnh, tên kèm variant title, giá). Không hiện option picker trên card.
+- Nested Options on card + Card behavior disable vì picker không áp dụng cho parent product.
+- Cấu hình option list vẫn giữ, không bị xóa.
+- Note: Each variant is already its own product card, so option pickers are not shown on the parent product.
+- Preview mockup: 2 card split (Navy / Red Wine) + variant title “· {value}”.
+- Production listing phải lấy variant thật của từng product, không hard-code 2 màu demo.
+- Mode này không tạo product Shopify mới; chỉ đổi presentation listing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADM-11
+Mockup: #variantAsProductToggle + .preview-split</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Options on card — list / add / remove
+- Bảng: # (presentation order), Option, Display, Show, Remove.
+- Option cell: dropdown đổi mapping + caption “N values · {source}” (+ metafield key nếu có).
+- Display: Image swatch / Color swatch / Text button / Not shown.
+- Show toggle. Display = Not shown → shown=false. Bật Show khi đang Not shown → gán default display theo data (có ảnh → Image swatch, có màu → Color swatch, không thì Text button).
+- Drag &amp; drop row đổi presentationOrder. Drag không hợp lệ: giữ thứ tự cũ.
+- Đổi option mapping trên row: không trùng key đã dùng; nếu Image swatch mà option mới không có ảnh → fallback defaultDisplay.
+- Remove (×): gỡ option khỏi card config; source catalog trở lại dropdown Add.
+- Include all: thêm mọi catalog option/metafield chưa có (không auto-thêm custom), set shown=true và display mặc định nếu đang Not shown.
+- Exclude all: mọi row shown=false, display=Not shown; không xóa row.
+- Add variant:
+  +) Shopify product option — chọn option chưa dùng.
+  +) Product metafield — chọn metafield chưa dùng.
+  +) Create custom option — nhập Option name, tạo display-only. Tên trống thì focus input, không add.
+- Empty: All available product options / metafields are already on the card.
+- Option catalog bị xóa sau sync: Needs attention hoặc ẩn, không render config rỗng trên storefront.
+- Data sync lỗi: giữ last known configuration.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADM-02 / ADM-03 / ADM-04 / LOG-01
+Sample mockup: Color shown Image swatch; Size &amp; Material Not shown. Catalog còn Style, Finish, Pattern, Length, Pack size, Fabric family.</t>
   </si>
   <si>
     <t xml:space="preserve">Display type
-- Merchant chọn: Image swatch, Color swatch, Text button, Dropdown, Not shown.
-- Default là suggestion theo dữ liệu (ảnh/màu có sẵn), merchant được override.
-- Không suy luận cứng theo tên option (không ép Color = swatch, Size = text).
+- Merchant chọn trên Quick setup: Image swatch, Color swatch, Text button, Not shown.
+- Default suggestion theo dữ liệu (ảnh/màu có sẵn), merchant override. Không ép theo tên option.
 - Thiếu ảnh/màu: fallback Text button hoặc value label. Không render thumbnail rỗng.
-- Display type = Not shown tương đương disable option khỏi card.
-- Đổi display type chỉ đổi presentation, không reset enabled / order / các option khác.</t>
+- Display type = Not shown tương đương ẩn option khỏi card.
+- Đổi display type chỉ đổi presentation, không reset order / các option khác.
+- Dropdown display type không nằm trong mockup Quick setup hiện tại — không spec UI admin cho release này.</t>
   </si>
   <si>
     <t xml:space="preserve">ADM-05</t>
   </si>
   <si>
     <t xml:space="preserve">Swatch shape
-- Circle / Square / Rounded.
-- Chỉ áp dụng Color swatch và Image swatch. Text button và Dropdown không bị ảnh hưởng.
+- Circle / Square / Rounded. Card-level, label Swatch shape.
+- Chỉ áp dụng Color swatch và Image swatch. Text button không bị ảnh hưởng.
 - Shape không hợp lệ: fallback Circle.</t>
   </si>
   <si>
@@ -195,33 +225,35 @@
   </si>
   <si>
     <t xml:space="preserve">Image source (Image swatch)
-- Thứ tự ưu tiên: option value image → variant featured image → manual image.
-- Swatch thumbnail lấy theo source đã chọn.
-- Ảnh product chính trên card chỉ đổi khi resolve được variant/combination hợp lệ.
+- Production nên ưu tiên: option value image → variant featured image → manual image.
+- Control Image source không còn trên Quick setup; chỉ còn legacy editor ẩn.
+- Swatch thumbnail lấy theo source đã chọn khi production hỗ trợ.
+- Ảnh product chính trên card chỉ đổi khi resolve được variant/combination hợp lệ (và click behavior = Update image and link).
 - Image swatch là presentation của value, không phải product media chính.</t>
   </si>
   <si>
-    <t xml:space="preserve">ADM-07 / LOG-03</t>
+    <t xml:space="preserve">ADM-07 / LOG-03 — control UI không nằm MVP Quick setup</t>
   </si>
   <si>
     <t xml:space="preserve">Click behavior và variant resolution
-- Update image and link: chỉ chạy khi app resolve được combination/variant khớp toàn bộ selected options.
-- Open Quick Add: chỉ khi resolve được variant; nếu không → fallback Open PDP.
-- Open PDP: luôn mở product page, không yêu cầu resolve xong trên card.
-- Selected state lưu theo source option id/name, ví dụ {Finish: Matte, Pack Size: 2 pack}.
-- Khách được chọn option theo thứ tự bất kỳ. Availability của option còn lại tính lại theo selection hiện tại (dynamic, không static).
-- Không match combination: giữ nguyên card, disable/grey/hide value xung đột, không đổi ảnh/giá/link sai variant.
-- Value không hợp lệ: bỏ selection đó, giữ trạng thái trước.
-- Khi combination hợp lệ: cập nhật ảnh, price, compare-at price và product link. Thiếu media → product featured image.</t>
+- Chỉ áp dụng khi Enable custom ON và variantAsProduct OFF.
+- Update image and link: chỉ chạy khi app resolve được combination/variant khớp selected options (source product_option).
+- Open quick add: chỉ khi resolve được variant; nếu không → fallback Open product page.
+- Open product page: luôn mở PDP, không yêu cầu resolve xong trên card.
+- Selected state lưu theo source key, ví dụ {Color: Navy, Size: S}.
+- Khách chọn option theo thứ tự bất kỳ. Availability option còn lại tính lại theo selection (dynamic).
+- Không match combination: giữ nguyên card, grey/hide/cross value xung đột, không đổi ảnh/giá/link sai variant.
+- Custom option và metafield không tự resolve SKU mới. Click custom chỉ đổi selected UI trên card; không invent variant mua được.
+- Khi combination hợp lệ: cập nhật ảnh, price, compare-at, product link. Thiếu media → product featured image.</t>
   </si>
   <si>
     <t xml:space="preserve">ADM-08 / VAR-01..04</t>
   </si>
   <si>
     <t xml:space="preserve">Overflow
-- Show +N more (single line): đo width thật của card; render các value vừa chỗ; luôn chừa chỗ cho badge +N; không wrap; không cắt giữa text — ẩn nguyên chip.
+- Show +N more (single line): đo width thật của card; render value vừa chỗ; luôn chừa chỗ badge +N; không wrap; không cắt giữa text — ẩn nguyên chip/swatch.
 - Không dùng số lượng value cố định cho mọi viewport.
-- Horizontal scroll: nowrap + overflow-x; hiện đủ value; không hiện +N; không làm tăng chiều cao card.
+- Horizontal scroll: nowrap + overflow-x; hiện đủ value; không hiện +N; không tăng chiều cao card.
 - Mục tiêu: tránh mobile card nhảy dòng / breakout, và lỗi XL / Wool bị cắt.</t>
   </si>
   <si>
@@ -229,64 +261,69 @@
   </si>
   <si>
     <t xml:space="preserve">Unavailable handling
-- Grey out / Hide / Cross out áp dụng cho value không mua được, tính từ variant data thật sau khi có selected options hiện tại.
-- Admin không nhập combination thủ công và preview không phải source of truth cho availability.
-- Khi selection đổi, availability các option còn lại được tính lại.
-- Nếu setting = Hide và mọi value của một option đều unavailable: ẩn cả option row, không để khung rỗng.
-- Sold-out toàn product: giữ sold-out state của theme.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADM-10 / AVA-01 / AVA-02
-Preview mockup hiện chưa inject availability scenario giả — đúng hướng.</t>
+- Grey out / Hide / Cross out áp dụng cho value không mua được, tính từ variant data thật sau selected options hiện tại.
+- Admin không nhập combination thủ công. Preview không phải source of truth cho availability.
+- Nếu Hide và mọi value của một option đều unavailable: ẩn cả option row, không để khung rỗng.
+- Sold-out toàn product: giữ sold-out state của theme.
+- Custom option không có inventory Shopify: không giả sold-out từ custom values.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADM-10 / AVA-01 / AVA-02</t>
   </si>
   <si>
     <t xml:space="preserve">Preview fidelity
-- Preview phản ánh: layout, display type, order, overflow, shape, option visibility.
-- Preview dùng sample product (Essential Oversized T-Shirt) để demo presentation.
-- Preview không được tạo availability scenario giả. Production luôn lấy variant data thật.
-- Nếu chưa có dữ liệu variant thật, preview chỉ là presentation sample, không phải source of truth.</t>
+- Preview phản ánh: Enable custom, variant-as-product, layout, display type, order, overflow, shape, option visibility.
+- Mode picker: 1 card Essential Oversized T-Shirt + option rows + selection note “Selected: …”.
+- Mode variant-as-product: preview-split 2 card, variant title, không option row. Note: Each variant is listed as its own product card in the grid.
+- Không còn Desktop / Mobile toggle trên mockup hiện tại.
+- Preview không tạo availability scenario giả. Production luôn lấy variant data thật.</t>
   </si>
   <si>
     <t xml:space="preserve">LOG-06</t>
   </si>
   <si>
     <t xml:space="preserve">Responsive
-- Desktop: render mọi option enabled; row không wrap ngoài overflow mode; width đo theo card thật, không theo viewport cố định.
-- Mobile: card co theo container; option row one-line hoặc scroll; không overflow toàn màn hình.
-- Không có setting riêng Mobile maximum. Mọi option enabled vẫn render theo overflow mode.
+- Desktop: layout 2 cột settings + sticky preview. Mọi option shown vẫn render theo overflow mode.
+- Mobile (&lt;900px): 1 cột, preview dưới settings; option row one-line hoặc scroll; không overflow toàn màn hình.
+- Không có setting Mobile maximum / max variant sets.
 - Card quá hẹp vẫn dùng +N/scroll, không phá product grid.</t>
   </si>
   <si>
-    <t xml:space="preserve">RES-01 / RES-02 — đã bỏ max variant sets trên card</t>
+    <t xml:space="preserve">RES-01 / RES-02</t>
   </si>
   <si>
     <t xml:space="preserve">Validation khi Save
-- VAL-01 Duplicate mapping: chặn Save nếu cùng source option nằm ở hai set. Không silently overwrite.
-- VAL-02 Missing source: Needs attention; không render config rỗng; fallback tắt set lỗi, giữ set còn hợp lệ.
-- VAL-03 Native Shopify swatch: cảnh báo nguy cơ hai lớp swatch (theme/category metafield). Merchant confirm ownership hoặc disable một renderer. Không tự render đúp.
-- VAL-04 Save feedback: hiện saved state nếu valid; error summary nếu invalid. Network lỗi: giữ draft local, cho retry.</t>
+- VAL-01 Duplicate mapping: chặn Save nếu cùng product option / metafield nằm ở hai row. Không silently overwrite.
+- VAL-02 Missing source: Needs attention; không render config rỗng; fallback tắt row lỗi, giữ row còn hợp lệ.
+- VAL-03 Native Shopify swatch: cảnh báo hai lớp swatch. Merchant confirm ownership hoặc disable một renderer. Không tự render đúp.
+- VAL-04 Save feedback: hiện “Changes saved” nếu valid; error summary nếu invalid. Network lỗi: giữ draft local, cho retry.
+- VAL-05 Custom option name trống: không add, không Save custom rỗng.
+- VAL-06 Custom/metafield không được persist như Shopify option mới.</t>
   </si>
   <si>
     <t xml:space="preserve">Must</t>
   </si>
   <si>
     <t xml:space="preserve">Exception / catalog không đồng nhất
-- EXC-01 Product không có option đã bật: ẩn set đó trên đúng card đó, không để label/chip/empty spacing. Set match khác vẫn render.
-- EXC-02 Hơn 3 option: vẫn render theo priority + overflow; không giới hạn data model = 3. Có thể warning admin nếu card quá tải (Should).
+- EXC-01 Product không có option đã bật: ẩn set đó trên đúng card, không empty spacing. Set match khác vẫn render.
+- EXC-02 Nhiều option: vẫn render theo order + overflow; không giới hạn data model = 3. Warning admin nếu card quá tải (Should).
 - EXC-03 Value dài, emoji, ký tự đặc biệt, duplicate label: escape text; +N/scroll; resolve bằng value id.
-- EXC-04 Theme/app khác: không chồng event handler, không duplicate control; namespace DOM/event; fallback PDP/Quick Add nếu card hook không tương thích.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EXC-01 Must / EXC-02 Should / EXC-03 Should / EXC-04 Must</t>
+- EXC-04 Theme/app khác: không chồng handler, không duplicate control; fallback PDP/Quick Add nếu card hook không tương thích.
+- EXC-05 Variant-as-product trên product không có variant: giữ 1 card product, không nhân bản giả.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EXC-01 Must / EXC-02 Should / EXC-03 Should / EXC-04 Must / EXC-05 Must</t>
   </si>
   <si>
     <t xml:space="preserve">Những gì không được làm
-- Không tạo option/value từ UI này.
+- Không tạo Shopify option / value / variant / SKU từ UI này.
+- Custom option chỉ display trên card, không invent combination mua được.
 - Không đổi Shopify option position khi reorder trên card.
 - Không dùng label làm unique key.
 - Không render empty frame / empty option row.
 - Không coi admin preview availability là production logic.
-- Không hard-code 3 option Color/Size/Material trong data model.</t>
+- Không hard-code 3 option Color/Size/Material trong data model.
+- Không hiện option picker khi variantAsProduct = true hoặc enableCustom = false.</t>
   </si>
   <si>
     <t xml:space="preserve">Feature</t>
@@ -305,72 +342,88 @@
   </si>
   <si>
     <t xml:space="preserve">Phạm vi UI
-- RQM này mô tả tab Product grid design → Product card variants trong Findter Filter &amp; Search.
-- Layout 2 cột: bên trái là Quick setup, bên phải là Preview card (sticky trên desktop).
-- Header app: logo TD + title Findter Filter &amp; Search.
+- App: Findter Filter &amp; Search. Nav item active: Filter &amp; Product Grid Design.
+- Page header: Filter &amp; product grid design. Subtitle: Configure how variant options appear on collection and search product cards.
+- Nút Save + save-status nằm trên page header (không còn Save changes cuối trang).
 - Tabs: Filter design (ngoài scope) / Product grid design (active).
-- Trên mobile (&lt;900px): xếp 1 cột, preview nằm dưới settings.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Settings.html — khối .quick-setup + .preview-card</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Feature toggle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Show variant options on product cards
-- Label: Enable variant options.
-- Helper: Show selectable options below the product price.
-- Control: toggle switch. Default trong mockup đang ON vì đây là màn demo; production default là OFF.
-- Khi OFF: ẩn toàn bộ option trên Preview; Options on card vẫn nhìn thấy để merchant cấu hình sẵn.
-- Help note dưới list option cập nhật theo option đang bật.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quick setup section 1</t>
+- Layout 2 cột: trái Product card variants (.quick-setup), phải Preview card sticky.
+- Mobile (&lt;900px): 1 cột, preview dưới settings.
+- Logo mockup: Fd.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Settings.html — .pg-head + .quick-setup + .preview-card</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Product card variants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khối Quick setup
+- Heading: Product card variants.
+- Intro: Turn this on to show variant options on product cards, then choose which options appear.
+- Row 1: Enable custom — toggle switch (#featureEnableToggle). Mockup default ON; production default OFF.
+- Row 2: Show each variant as its own product — toggle (#variantAsProductToggle) + desc Collection and search show one card per variant instead of one card per product. Default OFF.
+- Nested panel #variantSettings chứa Options on card + Card behavior. Disable khi Enable custom OFF hoặc variant-as-product ON (opacity ~0.42, pointer-events none), không ẩn.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quick setup enable rows</t>
   </si>
   <si>
     <t xml:space="preserve">Options on card</t>
   </si>
   <si>
-    <t xml:space="preserve">Danh sách option import từ product data
-Mỗi option row gồm:
-  +) số thứ tự presentation (1, 2, 3…)
-  +) Option name đậm + dòng phụ "N values detected"
-  +) dropdown Display type: Image swatch / Color swatch / Text button / Not shown
-  +) toggle enable
-- Merchant kéo thả row để đổi thứ tự. Preview đổi thứ tự option theo đó.
-- Chọn Display type = Not shown → tự tắt toggle của row đó.
-- Chọn display type khác Not shown → bật toggle.
-- Note động, ví dụ: "Color is shown on the product card. Other options remain available on the product page."
-- Không có nút Add option. Không có input tạo option thủ công.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sample mockup: Color (6 values), Size (6), Material (3)</t>
+    <t xml:space="preserve">Section Options on card
+- Head: Options on card + bulk actions Include all / Exclude all (link style).
+- Table columns: # | Option | Display | Show |
+Mỗi row:
+  +) số thứ tự presentation
+  +) dropdown Option (đổi mapping) + caption N values · Shopify product option / Product metafield / Custom option (+ metafield key)
+  +) dropdown Display: Image swatch / Color swatch / Text button / Not shown
+  +) toggle Show
+  +) nút × Remove
+- Kéo thả row để đổi thứ tự. Preview đổi theo.
+- Display = Not shown ⇔ Show OFF. Bật Show → default display theo data.
+- Add source row:
+  +) Option source: Shopify product option / Product metafield / Create custom option
+  +) Dropdown chọn option/metafield chưa dùng, hoặc text Option name khi custom
+  +) Nút Add variant
+- Source hint dưới dropdown:
+  +) product option: Use a Shopify product option already on variants (Color, Size…). Values stay in sync with catalog and can resolve to a purchasable variant.
+  +) metafield: Use a product metafield when the attribute is not a Shopify option. Good for display or filtering; it cannot create a new SKU by itself.
+  +) custom: Create a display-only option on the card. This does not create Shopify options or variants, so customers cannot buy a combination that does not exist.
+- Empty copy khi hết source: All available product options / metafields are already on the card.
+- Quick note động, ví dụ: Color is shown on the product card. Other options remain available on the product page.
+- Feature OFF: Product card variants is off. Enable it to show options on the card.
+- Variant-as-product ON: Each variant is already its own product card, so option pickers are not shown on the parent product.
+- Không option shown: No options are shown on the product card. Customers can choose them on the product page.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sample: Color Image swatch shown; Size, Material Not shown. Add catalog: Style, Finish, Pattern, Length, Pack size (custom.pack_size), Fabric family (custom.fabric_family).</t>
   </si>
   <si>
     <t xml:space="preserve">Card behavior</t>
   </si>
   <si>
-    <t xml:space="preserve">Khối setting dùng chung cho mọi option trên card:
+    <t xml:space="preserve">Khối setting dùng chung, label phụ Applies to all options:
   +) Swatch shape: Circle / Square / Rounded
   +) When a customer clicks an option: Update image and link / Open quick add / Open product page
 Advanced behavior (collapsed mặc định):
   +) When there are more values: Show +N more (single line) / Horizontal scroll
   +) Unavailable values: Grey out / Hide / Cross out
-- Đổi control này phải update Preview ngay, không cần Save trước.
+- Đổi control update Preview ngay, không cần Save trước.
 - Shape không đổi Text button.
-- Overflow áp dụng cả image swatch row và text chip row.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Khối Card behavior + details Advanced behavior</t>
+- Overflow áp dụng image swatch và text chip.
+- Cả khối nằm trong nested panel nên disable cùng Options on card.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Card behavior + details Advanced behavior</t>
   </si>
   <si>
     <t xml:space="preserve">Save</t>
   </si>
   <si>
-    <t xml:space="preserve">- Nút Save changes ở cuối trang.
-- Click: hiện "Changes saved" rồi tự ẩn (mockup).
-- Production: chặn Save nếu validation fail (duplicate mapping, missing source) và hiện error summary.
+    <t xml:space="preserve">- Nút Save trên page header, bên phải title.
+- Click mockup: hiện Changes saved rồi tự ẩn.
+- Production: chặn Save nếu validation fail (duplicate mapping, missing source, custom name trống) và hiện error summary.
 - Save không được hiện thành công nếu dữ liệu invalid.</t>
   </si>
   <si>
@@ -380,9 +433,9 @@
     <t xml:space="preserve">Legacy Variant Sets (ẩn)</t>
   </si>
   <si>
-    <t xml:space="preserve">Trong Settings.html vẫn còn editor Variant Sets cũ (max sets, hover-image source, mapping hex, interaction mode Quick select / Display only) nhưng đang bị ẩn (.legacy-settings).
-- Không đưa các control này vào MVP đang demo.
-- Không còn Mobile maximum / Max variant sets shown on card.
+    <t xml:space="preserve">Trong Settings.html vẫn còn editor Variant Sets cũ (max sets, hover-image source, mapping hex, interaction mode Quick select / Display only, Image source) nhưng đang bị ẩn (.legacy-settings).
+- Không đưa các control này vào MVP Quick setup đang demo.
+- Không còn Mobile maximum / Max variant sets shown on card / Desktop-Mobile preview toggle.
 - Nếu mở lại later, phải migrate rule cho khớp overflow +N, không cắt max cứng.</t>
   </si>
   <si>
@@ -395,19 +448,20 @@
     <t xml:space="preserve">Rule chung</t>
   </si>
   <si>
-    <t xml:space="preserve">Preview nằm cột phải, có Desktop / Mobile toggle.
-- Desktop: card full width cột preview.
-- Mobile: frame max-width ~210px, layout compact.
-Card sample:
-  +) ảnh sản phẩm + badge Sale
+    <t xml:space="preserve">Preview cột phải, heading Preview card. Không còn Desktop / Mobile toggle.
+Card sample (mode picker):
+  +) ảnh + badge Sale
   +) Name: Essential Oversized T-Shirt
   +) Vendor: Nike Sportswear
-  +) Price / compare-at / sale price
-  +) Option rows theo option đang enabled
-  +) Add to cart (chỉ để tạo cảm giác card, không phải flow checkout)
-- Preview không hiện drag handle, toggle Include/Exclude, hay control editor.
-- Note dưới preview: Desktop/Mobile shows all enabled options.
-- Selection note: "Selected: Navy / S" sau khi click.</t>
+  +) Price / compare-at / sale
+  +) Option groups theo option đang shown (label COLOR… + swatch/chip)
+  +) Selection note Selected: Navy / S
+  +) Add to cart (visual only)
+Mode variant-as-product: .preview-split, 2 card, name + variant title · Navy / · Red Wine, không option group.
+Note dưới preview:
+  +) picker: Preview shows the options currently enabled on the product card.
+  +) variant-as-product: Each variant is listed as its own product card in the grid.
+Preview không hiện drag handle, Include/Exclude, editor controls.</t>
   </si>
   <si>
     <t xml:space="preserve">Không dùng preview làm source of truth availability</t>
@@ -416,10 +470,11 @@
     <t xml:space="preserve">Visibility</t>
   </si>
   <si>
-    <t xml:space="preserve">- Feature OFF → ẩn mọi option group trên preview.
-- Option toggle OFF hoặc Display type = Not shown → ẩn đúng group đó.
-- Reorder option row → reorder group trên preview (Color / Size / Material).
-- Product không match một option: ẩn group đó, không để khoảng trống lớn.</t>
+    <t xml:space="preserve">- Enable custom OFF → ẩn mọi option group trên preview (vẫn 1 product card).
+- Variant-as-product ON → ẩn option group, hiện split variant cards.
+- Option Show OFF hoặc Display = Not shown → ẩn đúng group.
+- Reorder row → reorder group trên preview.
+- Product không match một option: ẩn group đó, không khoảng trống lớn.</t>
   </si>
   <si>
     <t xml:space="preserve">Overflow UI</t>
@@ -428,8 +483,8 @@
     <t xml:space="preserve">Show +N more (single line):
   +) row nowrap, hidden overflow
   +) chip/swatch không vừa thì ẩn nguyên item
-  +) badge +N hiện số item bị ẩn
-  +) thuật toán đo scrollWidth vs clientWidth cho text row (Size, Material)
+  +) badge +N = số item bị ẩn
+  +) đo scrollWidth vs clientWidth cho text row
 Horizontal scroll:
   +) hiện extra swatch/chip
   +) ẩn badge +N
@@ -442,154 +497,169 @@
     <t xml:space="preserve">Display type = Image swatch</t>
   </si>
   <si>
-    <t xml:space="preserve">Editor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- Default suggestion khi option có ảnh value/variant.
-- Dropdown Image source chỉ liên quan Image swatch: Option value image / Variant featured image / Upload manually.
-- Swatch shape áp dụng lên thumbnail.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Color trong mockup đang để Image swatch</t>
+    <t xml:space="preserve">Editor + Preview</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Default suggestion khi option có ảnh value/variant. Color sample mặc định Image swatch.
+- Swatch thumbnail; selected ring đậm; shape theo Swatch shape.
+- Click (Update image and link): đổi selected + đổi ảnh card theo image của value.
+- Không tự chọn option khác khi hover.
+- Thiếu ảnh: không ô trống — fallback color hoặc text.
+- Image source dropdown không nằm Quick setup.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Color trong mockup đang Image swatch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Display type = Color swatch</t>
   </si>
   <si>
     <t xml:space="preserve">Preview</t>
   </si>
   <si>
-    <t xml:space="preserve">- Swatch là thumbnail ảnh, selected có ring đậm.
-- Click value (nếu click behavior = Update image and link): đổi selected + đổi ảnh card theo data-image của swatch.
-- Không tự chọn option khác khi hover/click swatch.
-- Thiếu ảnh: không để ô trống — fallback color hoặc text.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Display type = Color swatch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- Swatch là hình màu (hex), cùng shape setting.
+    <t xml:space="preserve">- Swatch hình màu (hex), cùng shape.
 - Không lấy thumbnail ảnh.
-- Selected state giống Image swatch (ring).
-- Mapping màu production lấy từ dữ liệu Shopify / value; mockup dùng hex tĩnh (Navy #1C2B3A, Red Wine #8A1F1F…).</t>
+- Selected ring giống Image swatch.
+- Mapping production từ Shopify / value; mockup hex tĩnh (Navy #1C2B3A, Red Wine #8A1F1F…).</t>
   </si>
   <si>
     <t xml:space="preserve">Display type = Text button</t>
   </si>
   <si>
-    <t xml:space="preserve">- Chip chữ: S, M, L, XL / Cotton, Linen, Wool.
+    <t xml:space="preserve">- Chip chữ (S, M, L… / Cotton, Linen… / custom values).
 - One line + overflow +N hoặc horizontal scroll.
-- Chip dài không wrap xuống dòng, không cắt giữa chữ.
+- Chip dài không wrap, không cắt giữa chữ.
 - Unavailable: grey / strike / hide theo setting.</t>
   </si>
   <si>
-    <t xml:space="preserve">Size &amp; Material trong sample</t>
-  </si>
-  <si>
     <t xml:space="preserve">Validation UI</t>
   </si>
   <si>
     <t xml:space="preserve">Needs attention / native swatch</t>
   </si>
   <si>
-    <t xml:space="preserve">- Option source mất: badge Needs attention trên row, không cho persist config rỗng.
-- Detect theme/native Shopify swatch: warning duplicate two swatch layers. Merchant phải chọn 1 renderer.
-- Duplicate mapping: highlight row lỗi + chặn Save. Copy: báo option bị map trùng, không tự gộp.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VAL-01 / VAL-02 / VAL-03</t>
+    <t xml:space="preserve">- Option source mất: badge Needs attention trên row, không persist config rỗng.
+- Detect theme/native Shopify swatch: warning duplicate two swatch layers.
+- Duplicate mapping: highlight row + chặn Save.
+- Custom name trống khi Add: không tạo row.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VAL-01 / VAL-02 / VAL-03 / VAL-05</t>
   </si>
   <si>
     <t xml:space="preserve">1. Mục tiêu
-Xây dựng UI và behavior của variant options trên product card storefront (Collection / Search) khi merchant đã bật Enable variant options trong Findter Settings.
-Khách chọn option trên card để preview variant (ảnh/giá/link) hoặc đi tiếp Quick Add / PDP, mà không phá layout card.</t>
+Xây dựng UI và behavior product card storefront (Collection / Search) theo cấu hình Findter Settings.
+Hai mode:
+- Enable custom ON + variant-as-product OFF: khách chọn option trên card để preview variant (ảnh/giá/link) hoặc đi Quick Add / PDP, không phá layout card.
+- Variant-as-product ON: grid liệt kê mỗi variant như một product card riêng, không hiện option picker trên card.</t>
   </si>
   <si>
     <t xml:space="preserve">2. Phạm vi áp dụng
 - Collection page product grid và Search Result product card.
-- Hỗ trợ display type: Image swatch, Color swatch, Text button, Dropdown.
+- Display type trên card: Image swatch, Color swatch, Text button.
 - Không thay Variant Picker trên PDP. Option không show trên card vẫn chọn được trên PDP.
-- Compatible với Quick Add nếu resolve được variant.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Cấu trúc hiển thị trên card
+- Compatible với Quick Add nếu resolve được variant (chỉ product_option).
+- Custom option / metafield trên card là presentation; không tạo SKU mới.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Cấu trúc hiển thị — mode option picker
 Thứ tự từ trên xuống:
 - Product media + badge (Sale…)
 - Product name, vendor, price
-- Các option row theo presentationOrder của option đang enabled
-- CTA Add to cart / Quick add (theo theme/app, không do setting này vẽ lại toàn bộ card)
-Mỗi option row:
-- Label option (COLOR, SIZE, MATERIAL…)
-- Value controls theo display type
-Không render row nếu: feature off, option disabled, không có source, visible value count = 0, hoặc Hide hết value unavailable.</t>
+- Option rows theo presentationOrder của option đang shown
+- CTA Add to cart / Quick add (theme/app)
+Mỗi option row: label option (COLOR…) + value controls theo display type.
+Không render row nếu: Enable custom off, variant-as-product on, option not shown, không có source, visible value count = 0, hoặc Hide hết value unavailable.</t>
   </si>
   <si>
     <t xml:space="preserve">EXC-01</t>
   </si>
   <si>
-    <t xml:space="preserve">4. Logic selected options và combination
+    <t xml:space="preserve">4. Cấu trúc hiển thị — mode variant as product
+- Một card cho mỗi variant (không gộp về 1 product).
+- Name có thể kèm variant title (· Navy).
+- Ảnh / giá theo đúng variant đó.
+- Không render option picker trên card.
+- Product không có variant: 1 card, không nhân bản giả.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADM-11 / EXC-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. Logic selected options và combination (mode picker)
 - State theo option id, không hard-code color/size.
-- Chỉ update image, price, compare-at, product link khi match variant chứa đủ selected values.
+- Chỉ update image, price, compare-at, product link khi match variant chứa đủ selected product_option values.
 - Không match: giữ card, đánh dấu value xung đột theo unavailable style.
-- Availability là dynamic theo selection hiện tại.
-- Selection invalid: reset option cuối hoặc yêu cầu chọn lại, không add nhầm variant.
-- Unique key = option value id. Duplicate label vẫn resolve đúng id.</t>
+- Availability dynamic theo selection hiện tại.
+- Custom/metafield click không invent variant.
+- Unique key = value id. Duplicate label vẫn resolve đúng id.</t>
   </si>
   <si>
     <t xml:space="preserve">VAR-01..04</t>
   </si>
   <si>
-    <t xml:space="preserve">5. UI &amp; behavior theo Display type
-5.1 Image swatch
-- Thumbnail value; selected ring rõ; hover không tự đổi option khác.
-- Ảnh card chỉ đổi sau khi combination hợp lệ.
-5.2 Color swatch
-- Hình màu theo mapping; cùng shape Circle/Square/Rounded.
-5.3 Text button
-- Chip label; one-line overflow.
-5.4 Dropdown
-- Dùng khi nhiều value / merchant chọn; không phá chiều cao card quá mức (Should theo display type list).
-Click action (dùng chung):
+    <t xml:space="preserve">6. UI &amp; behavior theo Display type
+6.1 Image swatch: thumbnail; selected ring; hover không tự đổi option khác; ảnh card đổi sau combination hợp lệ.
+6.2 Color swatch: hình màu; shape Circle/Square/Rounded.
+6.3 Text button: chip label; one-line overflow.
+Click action card-level:
 - Update image and link
 - Open Quick Add (fallback PDP nếu không resolve)
 - Open product page</t>
   </si>
   <si>
-    <t xml:space="preserve">6. Overflow
+    <t xml:space="preserve">7. Overflow
 - +N single line: đo width card thật, chừa badge, ẩn nguyên chip, không wrap, không cắt giữa text (fix XL/Wool).
 - Horizontal scroll: đủ value, không +N, không tăng height card.
-- Desktop grid nhiều cột và mobile đều dùng cùng rule, chỉ khác container width.</t>
+- Desktop nhiều cột và mobile cùng rule, khác container width.</t>
   </si>
   <si>
     <t xml:space="preserve">LOG-04 / LOG-05 / RES-02</t>
   </si>
   <si>
-    <t xml:space="preserve">7. Unavailable values
+    <t xml:space="preserve">8. Unavailable values
 - Grey out / Hide / Cross out theo admin.
 - Tính từ imported variant data, không từ preview giả.
 - Hide hết value → ẩn cả option row.
-- Product sold out: theo theme sold-out, không vẽ control gây hiểu nhầm.</t>
+- Product sold out: theo theme sold-out.</t>
   </si>
   <si>
     <t xml:space="preserve">AVA-01 / AVA-02</t>
   </si>
   <si>
-    <t xml:space="preserve">8. Responsive
-- Desktop: mọi option enabled, không wrap ngoài overflow.
-- Mobile: card theo container; option one-line hoặc scroll; không breakout viewport; không nhảy height vì wrap.
-- Không có Mobile maximum riêng.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9. Compatibility
-- Không render đúp nếu theme/native Shopify swatch đã có trên card. Respect warning admin đã chốt.
+    <t xml:space="preserve">9. Responsive
+- Desktop: mọi option shown, không wrap ngoài overflow.
+- Mobile: card theo container; option one-line hoặc scroll; không breakout viewport.
+- Không có Mobile maximum riêng.
+- Variant-as-product: grid nhiều card hơn; card vẫn cùng template, không option row.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10. Compatibility
+- Không render đúp nếu theme/native Shopify swatch đã có trên card.
 - Namespace DOM/event, không chồng handler theme/filter app khác.
-- Card hook không tương thích → fallback PDP / Quick Add, không silent fail khiến khách chọn sai variant.</t>
+- Card hook không tương thích → fallback PDP / Quick Add, không silent fail.</t>
   </si>
   <si>
     <t xml:space="preserve">VAL-03 / EXC-04</t>
   </si>
   <si>
-    <t xml:space="preserve">10. Những gì không xuất hiện trên storefront card
-- Drag handle, admin toggle, Needs attention, mapping hex editor, Save.
+    <t xml:space="preserve">11. Những gì không xuất hiện trên storefront card
+- Drag handle, admin toggle, Include all / Exclude all, Add variant, Needs attention, mapping hex editor, Save.
 - Empty wrapper / empty option frame.
-- Option đang Not shown / disabled / không match product.</t>
+- Option đang Not shown / disabled / không match product.
+- Option picker khi variant-as-product ON hoặc Enable custom OFF.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Product Card Variant Options / Admin behavior</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Code UI/UX tham khảo: Settings.html
+Live mockup: https://hainx-bss.github.io/Settings/
+Format gốc: RDS_Findter_Merged_Filter_RQM.xlsx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI web tham khảo:
+https://hainx-bss.github.io/Settings/</t>
   </si>
 </sst>
 </file>
@@ -922,7 +992,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="18" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -945,7 +1015,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="94" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="224" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -959,46 +1029,63 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="112" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="B4" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="94" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="112" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="2"/>
       <c r="B5" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>15</v>
+      </c>
+      <c r="D5" s="2"/>
+    </row>
+    <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="2"/>
       <c r="B6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="D6" s="2"/>
+    </row>
+    <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1025,13 +1112,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>16</v>
+        <v>114</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>17</v>
+        <v>115</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>18</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1039,152 +1126,153 @@
     </row>
     <row r="3" customFormat="false" ht="22" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="164" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="272" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="160" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B5" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="80" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+    <row r="6" customFormat="false" ht="208" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B6" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="122" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+    <row r="7" customFormat="false" ht="272" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B7" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="178" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+    <row r="8" customFormat="false" ht="192" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B8" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="108" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+    <row r="9" customFormat="false" ht="208" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B9" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="108" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+    <row r="10" customFormat="false" ht="368" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B10" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="108" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+    <row r="11" customFormat="false" ht="160" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B11" s="2" t="s">
         <v>33</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="122" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="80" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="128" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B13" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="80" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
+    <row r="14" customFormat="false" ht="256" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B14" s="2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="206" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+    <row r="15" customFormat="false" ht="128" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B15" s="2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="108" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
+    <row r="16" customFormat="false" ht="128" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B16" s="2" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="136" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
+    <row r="17" customFormat="false" ht="144" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B17" s="2" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="108" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="s">
+    <row r="18" customFormat="false" ht="128" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B18" s="2" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="122" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
+    <row r="19" customFormat="false" ht="192" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B19" s="2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="136" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
+    <row r="20" customFormat="false" ht="192" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B20" s="2" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="136" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="s">
+    <row r="21" customFormat="false" ht="160" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="108" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2" t="s">
-        <v>54</v>
-      </c>
+      <c r="B21" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1205,7 +1293,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="18" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
@@ -1216,13 +1304,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>16</v>
+        <v>114</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>17</v>
+        <v>115</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>18</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1230,203 +1318,192 @@
     </row>
     <row r="3" customFormat="false" ht="22" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>55</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>57</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="122" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="160" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C4" s="2" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="208" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="122" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B5" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="C5" s="2" t="s">
+    </row>
+    <row r="6" customFormat="false" ht="528" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="C6" s="2" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="192" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C6" s="2" t="s">
+    </row>
+    <row r="7" customFormat="false" ht="192" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="C7" s="2" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B7" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C7" s="2" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="C8" s="2" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="80" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B8" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C8" s="2" t="s">
+    </row>
+    <row r="9" customFormat="false" ht="128" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="C9" s="2" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="94" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C9" s="2" t="s">
+    </row>
+    <row r="10" customFormat="false" ht="256" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="B10" s="2" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="192" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="C10" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C10" s="2" t="s">
+    </row>
+    <row r="11" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="C11" s="2" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B11" s="2" t="s">
+      <c r="D11" s="2"/>
+    </row>
+    <row r="12" customFormat="false" ht="160" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C12" s="2" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="136" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B12" s="2" t="s">
+      <c r="D12" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C12" s="2" t="s">
+    </row>
+    <row r="13" customFormat="false" ht="128" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="B13" s="2" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
+      <c r="C13" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="D13" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C13" s="2" t="s">
+    </row>
+    <row r="14" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="B14" s="2" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="80" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="B14" s="2" t="s">
+      <c r="C14" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>91</v>
-      </c>
+      <c r="D14" s="2"/>
     </row>
     <row r="15" customFormat="false" ht="80" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="2"/>
+    </row>
+    <row r="16" customFormat="false" ht="80" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
+      <c r="B16" s="2" t="s">
         <v>94</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>90</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>95</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>96</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="94" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -1448,7 +1525,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="18" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
@@ -1459,13 +1536,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>16</v>
+        <v>114</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>17</v>
+        <v>115</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>18</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1473,102 +1550,117 @@
     </row>
     <row r="3" customFormat="false" ht="22" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>55</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>57</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="94" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="144" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="94" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>97</v>
+      </c>
+      <c r="D4" s="2"/>
+    </row>
+    <row r="5" customFormat="false" ht="128" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="178" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>98</v>
+      </c>
+      <c r="D5" s="2"/>
+    </row>
+    <row r="6" customFormat="false" ht="160" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="136" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="112" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="220" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="144" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="94" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>103</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="160" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="80" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>105</v>
+      </c>
+      <c r="D9" s="2"/>
+    </row>
+    <row r="10" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="80" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="94" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>108</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>110</v>
+      </c>
+      <c r="D12" s="2"/>
+    </row>
+    <row r="13" customFormat="false" ht="80" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2" t="s">
-        <v>115</v>
-      </c>
+        <v>111</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="112" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D14" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>